<commit_message>
CV Coach scan 2026-08-30 (scan-jobs): 79 PM jobs scored, best 6/10 (Swan.io / Splio), none cleared 9.3 auto-prep bar
</commit_message>
<xml_diff>
--- a/applications/Job_Matches_Paris_ProductAI.xlsx
+++ b/applications/Job_Matches_Paris_ProductAI.xlsx
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1347"/>
+  <dimension ref="A1:M1370"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -61609,6 +61609,869 @@
         </is>
       </c>
     </row>
+    <row r="1348">
+      <c r="A1348" t="inlineStr"/>
+      <c r="B1348" t="n">
+        <v>5</v>
+      </c>
+      <c r="C1348" t="inlineStr">
+        <is>
+          <t>Senior Product Manager - Agentic &amp; ai Automation H/F</t>
+        </is>
+      </c>
+      <c r="D1348" t="inlineStr">
+        <is>
+          <t>Believe</t>
+        </is>
+      </c>
+      <c r="E1348" t="inlineStr">
+        <is>
+          <t>Paris - 75</t>
+        </is>
+      </c>
+      <c r="F1348" t="inlineStr"/>
+      <c r="G1348" t="inlineStr"/>
+      <c r="H1348" t="inlineStr"/>
+      <c r="I1348" t="inlineStr"/>
+      <c r="J1348" t="inlineStr"/>
+      <c r="K1348" t="inlineStr">
+        <is>
+          <t>https://www.hellowork.com/fr-fr/entreprises/believe-91896.html</t>
+        </is>
+      </c>
+      <c r="L1348" t="inlineStr">
+        <is>
+          <t>Strength: AI relevance. Gap: no target-sector bonus.</t>
+        </is>
+      </c>
+      <c r="M1348" t="inlineStr">
+        <is>
+          <t>Not yet applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="1349">
+      <c r="A1349" t="inlineStr"/>
+      <c r="B1349" t="n">
+        <v>5</v>
+      </c>
+      <c r="C1349" t="inlineStr">
+        <is>
+          <t>Product Manager B2b H/F</t>
+        </is>
+      </c>
+      <c r="D1349" t="inlineStr">
+        <is>
+          <t>Bloomays</t>
+        </is>
+      </c>
+      <c r="E1349" t="inlineStr">
+        <is>
+          <t>Paris - 75</t>
+        </is>
+      </c>
+      <c r="F1349" t="inlineStr"/>
+      <c r="G1349" t="inlineStr"/>
+      <c r="H1349" t="inlineStr"/>
+      <c r="I1349" t="inlineStr"/>
+      <c r="J1349" t="inlineStr"/>
+      <c r="L1349" t="inlineStr">
+        <is>
+          <t>Strength: finance/domain overlap. Gap: no target-sector bonus.</t>
+        </is>
+      </c>
+      <c r="M1349" t="inlineStr">
+        <is>
+          <t>Not yet applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="1350">
+      <c r="A1350" t="inlineStr"/>
+      <c r="B1350" t="n">
+        <v>4</v>
+      </c>
+      <c r="C1350" t="inlineStr">
+        <is>
+          <t>Product Manager - Sales ai H/F</t>
+        </is>
+      </c>
+      <c r="D1350" t="inlineStr">
+        <is>
+          <t>Alan</t>
+        </is>
+      </c>
+      <c r="E1350" t="inlineStr">
+        <is>
+          <t>Paris - 75</t>
+        </is>
+      </c>
+      <c r="F1350" t="inlineStr"/>
+      <c r="G1350" t="inlineStr"/>
+      <c r="H1350" t="inlineStr"/>
+      <c r="I1350" t="inlineStr"/>
+      <c r="J1350" t="inlineStr"/>
+      <c r="K1350" t="inlineStr">
+        <is>
+          <t>https://www.hellowork.com/fr-fr/entreprises/alan-116878.html</t>
+        </is>
+      </c>
+      <c r="L1350" t="inlineStr">
+        <is>
+          <t>Strength: seniority fit. Gap: no named recruiter.</t>
+        </is>
+      </c>
+      <c r="M1350" t="inlineStr">
+        <is>
+          <t>Not yet applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="1351">
+      <c r="A1351" t="inlineStr"/>
+      <c r="B1351" t="n">
+        <v>4</v>
+      </c>
+      <c r="C1351" t="inlineStr">
+        <is>
+          <t>Technical Product Manager - Product Owner H/F</t>
+        </is>
+      </c>
+      <c r="D1351" t="inlineStr">
+        <is>
+          <t>Dev &amp; Connect</t>
+        </is>
+      </c>
+      <c r="E1351" t="inlineStr">
+        <is>
+          <t>Paris - 75</t>
+        </is>
+      </c>
+      <c r="F1351" t="inlineStr"/>
+      <c r="G1351" t="inlineStr"/>
+      <c r="H1351" t="inlineStr"/>
+      <c r="I1351" t="inlineStr"/>
+      <c r="J1351" t="inlineStr"/>
+      <c r="L1351" t="inlineStr">
+        <is>
+          <t>Strength: AI relevance. Gap: no target-sector bonus.</t>
+        </is>
+      </c>
+      <c r="M1351" t="inlineStr">
+        <is>
+          <t>Not yet applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="1352">
+      <c r="A1352" t="inlineStr"/>
+      <c r="B1352" t="n">
+        <v>4</v>
+      </c>
+      <c r="C1352" t="inlineStr">
+        <is>
+          <t>Product Manager IA H/F</t>
+        </is>
+      </c>
+      <c r="D1352" t="inlineStr">
+        <is>
+          <t>5 Degrés</t>
+        </is>
+      </c>
+      <c r="E1352" t="inlineStr">
+        <is>
+          <t>Paris - 75</t>
+        </is>
+      </c>
+      <c r="F1352" t="inlineStr"/>
+      <c r="G1352" t="inlineStr"/>
+      <c r="H1352" t="inlineStr"/>
+      <c r="I1352" t="inlineStr"/>
+      <c r="J1352" t="inlineStr"/>
+      <c r="L1352" t="inlineStr">
+        <is>
+          <t>Strength: AI relevance. Gap: no target-sector bonus.</t>
+        </is>
+      </c>
+      <c r="M1352" t="inlineStr">
+        <is>
+          <t>Not yet applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="1353">
+      <c r="A1353" t="inlineStr"/>
+      <c r="B1353" t="n">
+        <v>4</v>
+      </c>
+      <c r="C1353" t="inlineStr">
+        <is>
+          <t>Product Manager Data H/F</t>
+        </is>
+      </c>
+      <c r="D1353" t="inlineStr">
+        <is>
+          <t>Yunik</t>
+        </is>
+      </c>
+      <c r="E1353" t="inlineStr">
+        <is>
+          <t>Paris - 75</t>
+        </is>
+      </c>
+      <c r="F1353" t="inlineStr"/>
+      <c r="G1353" t="inlineStr"/>
+      <c r="H1353" t="inlineStr"/>
+      <c r="I1353" t="inlineStr"/>
+      <c r="J1353" t="inlineStr"/>
+      <c r="L1353" t="inlineStr">
+        <is>
+          <t>Strength: finance/domain overlap. Gap: no target-sector bonus.</t>
+        </is>
+      </c>
+      <c r="M1353" t="inlineStr">
+        <is>
+          <t>Not yet applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="1354">
+      <c r="A1354" t="inlineStr"/>
+      <c r="B1354" t="n">
+        <v>4</v>
+      </c>
+      <c r="C1354" t="inlineStr">
+        <is>
+          <t>Product Manager Officer H/F</t>
+        </is>
+      </c>
+      <c r="D1354" t="inlineStr">
+        <is>
+          <t>Caisse des Dépôts et Consignations (CDC)</t>
+        </is>
+      </c>
+      <c r="E1354" t="inlineStr">
+        <is>
+          <t>Paris 13e - 75</t>
+        </is>
+      </c>
+      <c r="F1354" t="inlineStr"/>
+      <c r="G1354" t="inlineStr"/>
+      <c r="H1354" t="inlineStr"/>
+      <c r="I1354" t="inlineStr"/>
+      <c r="J1354" t="inlineStr"/>
+      <c r="L1354" t="inlineStr">
+        <is>
+          <t>Strength: finance/domain overlap. Gap: no target-sector bonus.</t>
+        </is>
+      </c>
+      <c r="M1354" t="inlineStr">
+        <is>
+          <t>Not yet applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="1355">
+      <c r="A1355" t="inlineStr"/>
+      <c r="B1355" t="n">
+        <v>4</v>
+      </c>
+      <c r="C1355" t="inlineStr">
+        <is>
+          <t>Senior Product Manager - User And Lifecycle Analytics H/F</t>
+        </is>
+      </c>
+      <c r="D1355" t="inlineStr">
+        <is>
+          <t>Contentsquare</t>
+        </is>
+      </c>
+      <c r="E1355" t="inlineStr">
+        <is>
+          <t>Paris - 75</t>
+        </is>
+      </c>
+      <c r="F1355" t="inlineStr"/>
+      <c r="G1355" t="inlineStr"/>
+      <c r="H1355" t="inlineStr"/>
+      <c r="I1355" t="inlineStr"/>
+      <c r="J1355" t="inlineStr"/>
+      <c r="K1355" t="inlineStr">
+        <is>
+          <t>https://www.hellowork.com/fr-fr/entreprises/contentsquare-97142.html</t>
+        </is>
+      </c>
+      <c r="L1355" t="inlineStr">
+        <is>
+          <t>Strength: seniority fit. Gap: limited AI-specific scope.</t>
+        </is>
+      </c>
+      <c r="M1355" t="inlineStr">
+        <is>
+          <t>Not yet applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="1356">
+      <c r="A1356" t="inlineStr"/>
+      <c r="B1356" t="n">
+        <v>4</v>
+      </c>
+      <c r="C1356" t="inlineStr">
+        <is>
+          <t>Responsable du pôle Product Management - Secteur Energie F/H</t>
+        </is>
+      </c>
+      <c r="D1356" t="inlineStr">
+        <is>
+          <t>Groupe Talents Handicap</t>
+        </is>
+      </c>
+      <c r="E1356" t="inlineStr">
+        <is>
+          <t>Nanterre</t>
+        </is>
+      </c>
+      <c r="F1356" t="inlineStr"/>
+      <c r="G1356" t="inlineStr"/>
+      <c r="H1356" t="inlineStr"/>
+      <c r="I1356" t="inlineStr"/>
+      <c r="J1356" t="inlineStr"/>
+      <c r="K1356" t="inlineStr">
+        <is>
+          <t>https://www.glassdoor.fr/job-listing/responsable-du-pôle-product-management-secteur-energie-fh-groupe-talents-handicap-JV_IC3019245_KO0,57_KE58,81.htm?jl=1010245287964</t>
+        </is>
+      </c>
+      <c r="L1356" t="inlineStr">
+        <is>
+          <t>Strength: seniority fit. Gap: no target-sector bonus.</t>
+        </is>
+      </c>
+      <c r="M1356" t="inlineStr">
+        <is>
+          <t>Not yet applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="1357">
+      <c r="A1357" t="inlineStr"/>
+      <c r="B1357" t="n">
+        <v>3</v>
+      </c>
+      <c r="C1357" t="inlineStr">
+        <is>
+          <t>Product Manager Data &amp; ai Platform H/F</t>
+        </is>
+      </c>
+      <c r="D1357" t="inlineStr">
+        <is>
+          <t>Wold</t>
+        </is>
+      </c>
+      <c r="E1357" t="inlineStr">
+        <is>
+          <t>Paris - 75</t>
+        </is>
+      </c>
+      <c r="F1357" t="inlineStr"/>
+      <c r="G1357" t="inlineStr"/>
+      <c r="H1357" t="inlineStr"/>
+      <c r="I1357" t="inlineStr"/>
+      <c r="J1357" t="inlineStr"/>
+      <c r="L1357" t="inlineStr">
+        <is>
+          <t>Strength: seniority fit. Gap: no target-sector bonus.</t>
+        </is>
+      </c>
+      <c r="M1357" t="inlineStr">
+        <is>
+          <t>Not yet applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="1358">
+      <c r="A1358" t="inlineStr"/>
+      <c r="B1358" t="n">
+        <v>3</v>
+      </c>
+      <c r="C1358" t="inlineStr">
+        <is>
+          <t>Senior Product Manager - ai H/F</t>
+        </is>
+      </c>
+      <c r="D1358" t="inlineStr">
+        <is>
+          <t>Front</t>
+        </is>
+      </c>
+      <c r="E1358" t="inlineStr">
+        <is>
+          <t>Paris - 75</t>
+        </is>
+      </c>
+      <c r="F1358" t="inlineStr"/>
+      <c r="G1358" t="inlineStr"/>
+      <c r="H1358" t="inlineStr"/>
+      <c r="I1358" t="inlineStr"/>
+      <c r="J1358" t="inlineStr"/>
+      <c r="K1358" t="inlineStr">
+        <is>
+          <t>https://www.hellowork.com/fr-fr/entreprises/front-107796.html</t>
+        </is>
+      </c>
+      <c r="L1358" t="inlineStr">
+        <is>
+          <t>Strength: seniority fit. Gap: no target-sector bonus.</t>
+        </is>
+      </c>
+      <c r="M1358" t="inlineStr">
+        <is>
+          <t>Not yet applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="1359">
+      <c r="A1359" t="inlineStr"/>
+      <c r="B1359" t="n">
+        <v>3</v>
+      </c>
+      <c r="C1359" t="inlineStr">
+        <is>
+          <t>Dicom 75 - Responsable de l'Unité Produit - Head Of Product Sic H/F</t>
+        </is>
+      </c>
+      <c r="D1359" t="inlineStr">
+        <is>
+          <t>Service Public</t>
+        </is>
+      </c>
+      <c r="E1359" t="inlineStr">
+        <is>
+          <t>Paris - 75</t>
+        </is>
+      </c>
+      <c r="F1359" t="inlineStr"/>
+      <c r="G1359" t="inlineStr"/>
+      <c r="H1359" t="inlineStr"/>
+      <c r="I1359" t="inlineStr"/>
+      <c r="J1359" t="inlineStr"/>
+      <c r="L1359" t="inlineStr">
+        <is>
+          <t>Strength: seniority fit. Gap: no target-sector bonus.</t>
+        </is>
+      </c>
+      <c r="M1359" t="inlineStr">
+        <is>
+          <t>Not yet applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="1360">
+      <c r="A1360" t="inlineStr"/>
+      <c r="B1360" t="n">
+        <v>3</v>
+      </c>
+      <c r="C1360" t="inlineStr">
+        <is>
+          <t>Senior Data Product Manager H/F</t>
+        </is>
+      </c>
+      <c r="D1360" t="inlineStr">
+        <is>
+          <t>LittleBig Connection (part of Mantu)</t>
+        </is>
+      </c>
+      <c r="E1360" t="inlineStr">
+        <is>
+          <t>Paris - 75</t>
+        </is>
+      </c>
+      <c r="F1360" t="inlineStr"/>
+      <c r="G1360" t="inlineStr"/>
+      <c r="H1360" t="inlineStr"/>
+      <c r="I1360" t="inlineStr"/>
+      <c r="J1360" t="inlineStr"/>
+      <c r="L1360" t="inlineStr">
+        <is>
+          <t>Strength: seniority fit. Gap: no target-sector bonus.</t>
+        </is>
+      </c>
+      <c r="M1360" t="inlineStr">
+        <is>
+          <t>Not yet applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="1361">
+      <c r="A1361" t="inlineStr"/>
+      <c r="B1361" t="n">
+        <v>2</v>
+      </c>
+      <c r="C1361" t="inlineStr">
+        <is>
+          <t>Product Manager Discovery IA H/F</t>
+        </is>
+      </c>
+      <c r="D1361" t="inlineStr">
+        <is>
+          <t>Wold</t>
+        </is>
+      </c>
+      <c r="E1361" t="inlineStr">
+        <is>
+          <t>Paris - 75</t>
+        </is>
+      </c>
+      <c r="F1361" t="inlineStr"/>
+      <c r="G1361" t="inlineStr"/>
+      <c r="H1361" t="inlineStr"/>
+      <c r="I1361" t="inlineStr"/>
+      <c r="J1361" t="inlineStr"/>
+      <c r="L1361" t="inlineStr">
+        <is>
+          <t>Strength: seniority fit. Gap: no target-sector bonus.</t>
+        </is>
+      </c>
+      <c r="M1361" t="inlineStr">
+        <is>
+          <t>Not yet applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="1362">
+      <c r="A1362" t="inlineStr"/>
+      <c r="B1362" t="n">
+        <v>2</v>
+      </c>
+      <c r="C1362" t="inlineStr">
+        <is>
+          <t>Senior Technical Product Manager H/F</t>
+        </is>
+      </c>
+      <c r="D1362" t="inlineStr">
+        <is>
+          <t>Murex</t>
+        </is>
+      </c>
+      <c r="E1362" t="inlineStr">
+        <is>
+          <t>Paris - 75</t>
+        </is>
+      </c>
+      <c r="F1362" t="inlineStr"/>
+      <c r="G1362" t="inlineStr"/>
+      <c r="H1362" t="inlineStr"/>
+      <c r="I1362" t="inlineStr"/>
+      <c r="J1362" t="inlineStr"/>
+      <c r="K1362" t="inlineStr">
+        <is>
+          <t>https://www.hellowork.com/fr-fr/entreprises/murex-108701.html</t>
+        </is>
+      </c>
+      <c r="L1362" t="inlineStr">
+        <is>
+          <t>Strength: seniority fit. Gap: no target-sector bonus.</t>
+        </is>
+      </c>
+      <c r="M1362" t="inlineStr">
+        <is>
+          <t>Not yet applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="1363">
+      <c r="A1363" t="inlineStr"/>
+      <c r="B1363" t="n">
+        <v>2</v>
+      </c>
+      <c r="C1363" t="inlineStr">
+        <is>
+          <t>Product Manager Senior Mobile - CDI H/F</t>
+        </is>
+      </c>
+      <c r="D1363" t="inlineStr">
+        <is>
+          <t>SprintMob</t>
+        </is>
+      </c>
+      <c r="E1363" t="inlineStr">
+        <is>
+          <t>Paris - 75</t>
+        </is>
+      </c>
+      <c r="F1363" t="inlineStr"/>
+      <c r="G1363" t="inlineStr"/>
+      <c r="H1363" t="inlineStr"/>
+      <c r="I1363" t="inlineStr"/>
+      <c r="J1363" t="inlineStr"/>
+      <c r="L1363" t="inlineStr">
+        <is>
+          <t>Strength: seniority fit. Gap: no target-sector bonus.</t>
+        </is>
+      </c>
+      <c r="M1363" t="inlineStr">
+        <is>
+          <t>Not yet applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="1364">
+      <c r="A1364" t="inlineStr"/>
+      <c r="B1364" t="n">
+        <v>2</v>
+      </c>
+      <c r="C1364" t="inlineStr">
+        <is>
+          <t>Product Manager Poste de Travail Sécurisé H/F</t>
+        </is>
+      </c>
+      <c r="D1364" t="inlineStr">
+        <is>
+          <t>Service Public</t>
+        </is>
+      </c>
+      <c r="E1364" t="inlineStr">
+        <is>
+          <t>Paris 7e - 75</t>
+        </is>
+      </c>
+      <c r="F1364" t="inlineStr"/>
+      <c r="G1364" t="inlineStr"/>
+      <c r="H1364" t="inlineStr"/>
+      <c r="I1364" t="inlineStr"/>
+      <c r="J1364" t="inlineStr"/>
+      <c r="L1364" t="inlineStr">
+        <is>
+          <t>Strength: seniority fit. Gap: no target-sector bonus.</t>
+        </is>
+      </c>
+      <c r="M1364" t="inlineStr">
+        <is>
+          <t>Not yet applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="1365">
+      <c r="A1365" t="inlineStr"/>
+      <c r="B1365" t="n">
+        <v>1</v>
+      </c>
+      <c r="C1365" t="inlineStr">
+        <is>
+          <t>Chef - Cheffe de Produit ai Factory France H/F</t>
+        </is>
+      </c>
+      <c r="D1365" t="inlineStr">
+        <is>
+          <t>INRIA - Institut national de recherche en sciences et technologies du numérique</t>
+        </is>
+      </c>
+      <c r="E1365" t="inlineStr">
+        <is>
+          <t>Paris - 75</t>
+        </is>
+      </c>
+      <c r="F1365" t="inlineStr"/>
+      <c r="G1365" t="inlineStr"/>
+      <c r="H1365" t="inlineStr"/>
+      <c r="I1365" t="inlineStr"/>
+      <c r="J1365" t="inlineStr"/>
+      <c r="L1365" t="inlineStr">
+        <is>
+          <t>Strength: seniority fit. Gap: no target-sector bonus.</t>
+        </is>
+      </c>
+      <c r="M1365" t="inlineStr">
+        <is>
+          <t>Not yet applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="1366">
+      <c r="A1366" t="inlineStr"/>
+      <c r="B1366" t="n">
+        <v>1</v>
+      </c>
+      <c r="C1366" t="inlineStr">
+        <is>
+          <t>Product Manager Média H/F</t>
+        </is>
+      </c>
+      <c r="D1366" t="inlineStr">
+        <is>
+          <t>5 Degrés</t>
+        </is>
+      </c>
+      <c r="E1366" t="inlineStr">
+        <is>
+          <t>Paris - 75</t>
+        </is>
+      </c>
+      <c r="F1366" t="inlineStr"/>
+      <c r="G1366" t="inlineStr"/>
+      <c r="H1366" t="inlineStr"/>
+      <c r="I1366" t="inlineStr"/>
+      <c r="J1366" t="inlineStr"/>
+      <c r="L1366" t="inlineStr">
+        <is>
+          <t>Strength: seniority fit. Gap: no target-sector bonus.</t>
+        </is>
+      </c>
+      <c r="M1366" t="inlineStr">
+        <is>
+          <t>Not yet applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="1367">
+      <c r="A1367" t="inlineStr"/>
+      <c r="B1367" t="n">
+        <v>1</v>
+      </c>
+      <c r="C1367" t="inlineStr">
+        <is>
+          <t>Sgps - Product Manager H/F</t>
+        </is>
+      </c>
+      <c r="D1367" t="inlineStr">
+        <is>
+          <t>Agence Nationale de l'Habitat (ANAH)</t>
+        </is>
+      </c>
+      <c r="E1367" t="inlineStr">
+        <is>
+          <t>Paris - 75</t>
+        </is>
+      </c>
+      <c r="F1367" t="inlineStr"/>
+      <c r="G1367" t="inlineStr"/>
+      <c r="H1367" t="inlineStr"/>
+      <c r="I1367" t="inlineStr"/>
+      <c r="J1367" t="inlineStr"/>
+      <c r="L1367" t="inlineStr">
+        <is>
+          <t>Strength: seniority fit. Gap: no target-sector bonus.</t>
+        </is>
+      </c>
+      <c r="M1367" t="inlineStr">
+        <is>
+          <t>Not yet applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="1368">
+      <c r="A1368" t="inlineStr"/>
+      <c r="B1368" t="n">
+        <v>1</v>
+      </c>
+      <c r="C1368" t="inlineStr">
+        <is>
+          <t>Chef de Produit Applicatif IA H/F</t>
+        </is>
+      </c>
+      <c r="D1368" t="inlineStr">
+        <is>
+          <t>Service Public</t>
+        </is>
+      </c>
+      <c r="E1368" t="inlineStr">
+        <is>
+          <t>Paris 7e - 75</t>
+        </is>
+      </c>
+      <c r="F1368" t="inlineStr"/>
+      <c r="G1368" t="inlineStr"/>
+      <c r="H1368" t="inlineStr"/>
+      <c r="I1368" t="inlineStr"/>
+      <c r="J1368" t="inlineStr"/>
+      <c r="L1368" t="inlineStr">
+        <is>
+          <t>Strength: seniority fit. Gap: no target-sector bonus.</t>
+        </is>
+      </c>
+      <c r="M1368" t="inlineStr">
+        <is>
+          <t>Not yet applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="1369">
+      <c r="A1369" t="inlineStr"/>
+      <c r="B1369" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1369" t="inlineStr">
+        <is>
+          <t>Product Engineer Python - React - Nextjs H/F</t>
+        </is>
+      </c>
+      <c r="D1369" t="inlineStr">
+        <is>
+          <t>Zenior</t>
+        </is>
+      </c>
+      <c r="E1369" t="inlineStr">
+        <is>
+          <t>Paris - 75</t>
+        </is>
+      </c>
+      <c r="F1369" t="inlineStr"/>
+      <c r="G1369" t="inlineStr"/>
+      <c r="H1369" t="inlineStr"/>
+      <c r="I1369" t="inlineStr"/>
+      <c r="J1369" t="inlineStr"/>
+      <c r="L1369" t="inlineStr">
+        <is>
+          <t>Strength: seniority fit. Gap: no target-sector bonus.</t>
+        </is>
+      </c>
+      <c r="M1369" t="inlineStr">
+        <is>
+          <t>Not yet applied</t>
+        </is>
+      </c>
+    </row>
+    <row r="1370">
+      <c r="A1370" t="inlineStr"/>
+      <c r="B1370" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1370" t="inlineStr">
+        <is>
+          <t>CDI - Chef de Produit Prêt-À-Porter H/F</t>
+        </is>
+      </c>
+      <c r="D1370" t="inlineStr">
+        <is>
+          <t>Chanel</t>
+        </is>
+      </c>
+      <c r="E1370" t="inlineStr">
+        <is>
+          <t>Paris - 75</t>
+        </is>
+      </c>
+      <c r="F1370" t="inlineStr"/>
+      <c r="G1370" t="inlineStr"/>
+      <c r="H1370" t="inlineStr"/>
+      <c r="I1370" t="inlineStr"/>
+      <c r="J1370" t="inlineStr"/>
+      <c r="K1370" t="inlineStr">
+        <is>
+          <t>https://www.hellowork.com/fr-fr/entreprises/chanel-88659.html</t>
+        </is>
+      </c>
+      <c r="L1370" t="inlineStr">
+        <is>
+          <t>Strength: seniority fit. Gap: no target-sector bonus.</t>
+        </is>
+      </c>
+      <c r="M1370" t="inlineStr">
+        <is>
+          <t>Not yet applied</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:M91"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>